<commit_message>
Improved cash and recive view and to fix payment
</commit_message>
<xml_diff>
--- a/api/public/xlsx/inativos/clientes_inativos.xlsx
+++ b/api/public/xlsx/inativos/clientes_inativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="5">
   <si>
     <t>Cliente</t>
   </si>
@@ -30,15 +30,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>Teste 2</t>
-  </si>
-  <si>
-    <t>teste2@teste.com</t>
-  </si>
-  <si>
-    <t>Inativo</t>
   </si>
 </sst>
 </file>
@@ -378,7 +369,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -396,20 +387,6 @@
       </c>
       <c r="E1" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>12345678911</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
To fix validate CPF if = 1111111 or 4444444 and implemented configs customers
</commit_message>
<xml_diff>
--- a/api/public/xlsx/inativos/clientes_inativos.xlsx
+++ b/api/public/xlsx/inativos/clientes_inativos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
   <si>
     <t>Cliente</t>
   </si>
@@ -27,6 +27,15 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>Consumidor Padrão</t>
+  </si>
+  <si>
+    <t>Inativo</t>
+  </si>
+  <si>
+    <t>08805166901</t>
   </si>
 </sst>
 </file>
@@ -366,7 +375,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -381,6 +390,30 @@
       </c>
       <c r="D1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
To revise customers area
</commit_message>
<xml_diff>
--- a/api/public/xlsx/inativos/clientes_inativos.xlsx
+++ b/api/public/xlsx/inativos/clientes_inativos.xlsx
@@ -29,13 +29,13 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Consumidor Padrão</t>
+    <t>Sgbr Sistemas</t>
   </si>
   <si>
     <t>Inativo</t>
   </si>
   <si>
-    <t>08805166901</t>
+    <t>teste</t>
   </si>
 </sst>
 </file>
@@ -375,7 +375,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -396,23 +396,21 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
+      <c r="B2">
+        <v>17089484000190</v>
+      </c>
       <c r="D2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>41390805000176</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>